<commit_message>
4.0 test update using US values for SHELF and assorted other new non-elec sec files
</commit_message>
<xml_diff>
--- a/InputData/ccs/CCP/CO2 Capture Potentials.xlsx
+++ b/InputData/ccs/CCP/CO2 Capture Potentials.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CodeRepositories\eps-us\InputData\ccs\CCP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\ccs\CCP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6134759D-C76E-400C-8C70-93E8AFC83C7B}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB242916-3486-4863-B65A-1BC02A5C7437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21045" yWindow="1410" windowWidth="33360" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="CPPbES" sheetId="12" r:id="rId2"/>
     <sheet name="CPPbI" sheetId="13" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
   <si>
     <t>Source:</t>
   </si>
@@ -50,9 +50,6 @@
   </si>
   <si>
     <t>hard coal</t>
-  </si>
-  <si>
-    <t>natural gas nonpeaker</t>
   </si>
   <si>
     <t>nuclear</t>
@@ -290,6 +287,33 @@
   <si>
     <t>(We assume CO2 from "water and waste" is from waste collection trucks, not water treatment plants, which use almost entirely electricity.)</t>
   </si>
+  <si>
+    <t>natural gas steam turbine</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle</t>
+  </si>
+  <si>
+    <t>hard coal w CCS</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle w CCS</t>
+  </si>
+  <si>
+    <t>biomass w CCS</t>
+  </si>
+  <si>
+    <t>lignite w CCS</t>
+  </si>
+  <si>
+    <t>small modular reactor</t>
+  </si>
+  <si>
+    <t>hydrogen combustion turbine</t>
+  </si>
+  <si>
+    <t>hydrogen combined cycle</t>
+  </si>
 </sst>
 </file>
 
@@ -298,7 +322,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,6 +355,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -358,18 +389,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,9 +423,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -433,9 +463,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -468,26 +498,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -520,26 +533,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -736,12 +732,9 @@
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -749,97 +742,88 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>22</v>
+      <c r="A10" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="1"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="1"/>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="4"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="4"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="4"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="4"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="4"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
+      <c r="B22" s="6"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="10"/>
-      <c r="C22" s="2"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
+      <c r="B23" s="6"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="2"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -853,15 +837,15 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>21</v>
+      <c r="A1" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -869,20 +853,20 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -890,7 +874,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -898,7 +882,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -906,7 +890,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -914,7 +898,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -922,15 +906,15 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -938,31 +922,31 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -970,26 +954,90 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1012,19 +1060,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>21</v>
+      <c r="A1" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
         <v>33</v>
-      </c>
-      <c r="C1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1035,7 +1083,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1046,7 +1094,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1057,7 +1105,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1068,7 +1116,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -1079,7 +1127,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1090,7 +1138,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -1101,7 +1149,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1112,7 +1160,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -1123,7 +1171,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -1134,7 +1182,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -1145,7 +1193,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -1156,7 +1204,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1167,7 +1215,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -1178,7 +1226,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1189,7 +1237,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1200,7 +1248,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -1211,7 +1259,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -1222,7 +1270,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -1233,7 +1281,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -1244,7 +1292,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -1255,7 +1303,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B23">
         <v>1</v>
@@ -1266,7 +1314,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -1277,7 +1325,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -1288,7 +1336,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B26">
         <v>0</v>

</xml_diff>